<commit_message>
fix: unify report metadata, HTML, risk plots and KS Excel templates
</commit_message>
<xml_diff>
--- a/src/mars/reporting/template/mars_bin_report_linux.xlsx
+++ b/src/mars/reporting/template/mars_bin_report_linux.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\mars-risk\src\mars\analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\credit-risk\mars-risk\.artifacts\notebook-repair\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87CF90C6-A148-4043-B657-2517872A916C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{78252FC2-9B63-4C42-B28A-0C26A4539404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,11 +26,12 @@
   <pivotCaches>
     <pivotCache cacheId="8" r:id="rId9"/>
   </pivotCaches>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="56">
   <si>
     <t>y</t>
   </si>
@@ -210,6 +211,9 @@
   <si>
     <t>iv</t>
   </si>
+  <si>
+    <t>ks</t>
+  </si>
 </sst>
 </file>
 
@@ -353,1148 +357,7 @@
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="376">
-    <dxf>
-      <numFmt numFmtId="179" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
-      <alignment horizontal="left" vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <family val="2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <family val="2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <family val="2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
+  <dxfs count="167">
     <dxf>
       <font>
         <color theme="0"/>
@@ -1556,786 +419,6 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-        <charset val="134"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <family val="2"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="8"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="微软雅黑"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -2635,6 +718,797 @@
         <name val="微软雅黑"/>
         <family val="2"/>
         <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+        <charset val="134"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="179" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="9"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </font>
+      <alignment horizontal="left" vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="9"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="微软雅黑"/>
+        <charset val="134"/>
+        <scheme val="none"/>
       </font>
     </dxf>
   </dxfs>
@@ -2651,11 +1525,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="李士强" refreshedDate="46112.366218634263" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{52F49DAE-8B10-4720-B763-EACA38E5035D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="李士强" refreshedDate="46309.988869212961" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{52F49DAE-8B10-4720-B763-EACA38E5035D}">
   <cacheSource type="worksheet">
     <worksheetSource name="detail"/>
   </cacheSource>
-  <cacheFields count="21">
+  <cacheFields count="22">
     <cacheField name="y" numFmtId="0">
       <sharedItems containsNonDate="0" containsBlank="1" count="3">
         <m/>
@@ -2870,6 +1744,9 @@
         <m u="1"/>
       </sharedItems>
     </cacheField>
+    <cacheField name="ks" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
@@ -2903,6 +1780,7 @@
     <n v="0"/>
     <n v="0"/>
     <x v="0"/>
+    <m/>
   </r>
   <r>
     <x v="0"/>
@@ -2926,6 +1804,7 @@
     <n v="0"/>
     <n v="0"/>
     <x v="1"/>
+    <m/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -2933,7 +1812,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1E6BA4EB-C9E7-419D-885D-D579A93B5FA1}" name="分组透视" cacheId="8" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A5:G10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -3120,6 +1999,7 @@
         <item t="default"/>
       </items>
     </pivotField>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="2">
     <field x="1"/>
@@ -3179,35 +2059,35 @@
     <dataField name="iv" fld="18" baseField="1" baseItem="21" numFmtId="176"/>
   </dataFields>
   <formats count="38">
-    <format dxfId="353">
+    <format dxfId="166">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="352">
+    <format dxfId="165">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="351">
+    <format dxfId="164">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="350">
+    <format dxfId="163">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="349">
+    <format dxfId="162">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="348">
+    <format dxfId="161">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="347">
+    <format dxfId="160">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="346">
+    <format dxfId="159">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="345">
+    <format dxfId="158">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="1" count="0" selected="0"/>
@@ -3215,7 +2095,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="344">
+    <format dxfId="157">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3228,35 +2108,35 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="343">
+    <format dxfId="156">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="342">
+    <format dxfId="155">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="341">
+    <format dxfId="154">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="340">
+    <format dxfId="153">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="339">
+    <format dxfId="152">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="338">
+    <format dxfId="151">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="337">
+    <format dxfId="150">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="336">
+    <format dxfId="149">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="335">
+    <format dxfId="148">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="1" count="0" selected="0"/>
@@ -3264,7 +2144,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="334">
+    <format dxfId="147">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3277,19 +2157,19 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="333">
+    <format dxfId="146">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="332">
+    <format dxfId="145">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="331">
+    <format dxfId="144">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="330">
+    <format dxfId="143">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="329">
+    <format dxfId="142">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3302,19 +2182,19 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="328">
+    <format dxfId="141">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="327">
+    <format dxfId="140">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="326">
+    <format dxfId="139">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="325">
+    <format dxfId="138">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="324">
+    <format dxfId="137">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3327,7 +2207,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="323">
+    <format dxfId="136">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3340,7 +2220,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="322">
+    <format dxfId="135">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3353,7 +2233,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="321">
+    <format dxfId="134">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3366,7 +2246,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="320">
+    <format dxfId="133">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -3378,7 +2258,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="319">
+    <format dxfId="132">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -3390,7 +2270,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="318">
+    <format dxfId="131">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -3402,7 +2282,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="130">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3411,7 +2291,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="129">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -3439,7 +2319,7 @@
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C980371C-D21C-4C39-9001-37938B72DAD7}" name="数据透视表1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature">
   <location ref="A5:F6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -3610,11 +2490,12 @@
     <pivotField numFmtId="38" showAll="0"/>
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField dataField="1" numFmtId="176" showAll="0"/>
-    <pivotField dataField="1" numFmtId="176" showAll="0"/>
+    <pivotField numFmtId="176" showAll="0"/>
     <pivotField dataField="1" numFmtId="176" showAll="0"/>
     <pivotField dataField="1" numFmtId="176" showAll="0"/>
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -3651,31 +2532,31 @@
   <dataFields count="5">
     <dataField name="max(PSI) " fld="15" subtotal="max" baseField="1" baseItem="21" numFmtId="178"/>
     <dataField name="avg(IV) " fld="18" subtotal="average" baseField="1" baseItem="21" numFmtId="178"/>
-    <dataField name="avg(KS) " fld="16" subtotal="average" baseField="1" baseItem="21" numFmtId="178"/>
+    <dataField name="avg(KS) " fld="21" subtotal="average" baseField="1" baseItem="21" numFmtId="178"/>
     <dataField name="max(Lift) " fld="11" subtotal="max" baseField="1" baseItem="21" numFmtId="178"/>
     <dataField name="avg(AUC) " fld="17" subtotal="average" baseField="1" baseItem="21" numFmtId="178"/>
   </dataFields>
   <formats count="15">
-    <format dxfId="317">
+    <format dxfId="128">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="316">
+    <format dxfId="127">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="315">
+    <format dxfId="126">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="314">
+    <format dxfId="125">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="313">
+    <format dxfId="124">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="312">
+    <format dxfId="123">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3688,26 +2569,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="311">
+    <format dxfId="122">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="310">
+    <format dxfId="121">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="309">
+    <format dxfId="120">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="308">
+    <format dxfId="119">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="307">
+    <format dxfId="118">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="306">
+    <format dxfId="117">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="5">
@@ -3720,7 +2601,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="305">
+    <format dxfId="116">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -3729,7 +2610,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="304">
+    <format dxfId="115">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4" selected="0">
@@ -3741,7 +2622,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="303">
+    <format dxfId="114">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -3766,7 +2647,7 @@
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9AD699F8-3343-40F3-BC8D-6736B2D98F6C}" name="Missing" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="1"/>
@@ -3947,6 +2828,7 @@
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="38" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -3972,38 +2854,38 @@
     <dataField name="Missing rate" fld="9" baseField="1" baseItem="3" numFmtId="10"/>
   </dataFields>
   <formats count="10">
-    <format dxfId="302">
+    <format dxfId="113">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="301">
+    <format dxfId="112">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="300">
+    <format dxfId="111">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="299">
+    <format dxfId="110">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="298">
+    <format dxfId="109">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="297">
+    <format dxfId="108">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="296">
+    <format dxfId="107">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="295">
+    <format dxfId="106">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="294">
+    <format dxfId="105">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="293">
+    <format dxfId="104">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
@@ -4026,7 +2908,7 @@
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{67F0994E-2D0E-416D-B233-2A068F2B0705}" name="PSI" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -4207,6 +3089,7 @@
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -4232,63 +3115,63 @@
     <dataField name="PSI" fld="15" subtotal="max" baseField="1" baseItem="21" numFmtId="178"/>
   </dataFields>
   <formats count="17">
-    <format dxfId="292">
+    <format dxfId="103">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="291">
+    <format dxfId="102">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="290">
+    <format dxfId="101">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="289">
+    <format dxfId="100">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="288">
+    <format dxfId="99">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="287">
+    <format dxfId="98">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="286">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="285">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="284">
+    <format dxfId="95">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="283">
+    <format dxfId="94">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="282">
+    <format dxfId="93">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="281">
+    <format dxfId="92">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="280">
+    <format dxfId="91">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="279">
+    <format dxfId="90">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="278">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="277">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="276">
+    <format dxfId="87">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -4307,7 +3190,7 @@
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{140390A3-C4DA-44CD-8D5D-1808099448B4}" name="IV" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -4488,6 +3371,7 @@
     <pivotField dataField="1" numFmtId="176" showAll="0"/>
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -4513,63 +3397,63 @@
     <dataField name="IV" fld="18" baseField="1" baseItem="21" numFmtId="178"/>
   </dataFields>
   <formats count="17">
-    <format dxfId="275">
+    <format dxfId="86">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="274">
+    <format dxfId="85">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="273">
+    <format dxfId="84">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="272">
+    <format dxfId="83">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="271">
+    <format dxfId="82">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="270">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="269">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="268">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="267">
+    <format dxfId="78">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="266">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="265">
+    <format dxfId="76">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="264">
+    <format dxfId="75">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="263">
+    <format dxfId="74">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="262">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="261">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="260">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="259">
+    <format dxfId="70">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -4588,7 +3472,7 @@
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7B34FFD6-1423-4AE2-85E9-3157863EBEBF}" name="数据透视表2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -4764,11 +3648,12 @@
     <pivotField numFmtId="38" showAll="0"/>
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="176" showAll="0"/>
-    <pivotField dataField="1" numFmtId="176" showAll="0"/>
+    <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -4791,86 +3676,86 @@
     <pageField fld="5" item="116" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="KS" fld="16" subtotal="max" baseField="2" baseItem="0" numFmtId="178"/>
+    <dataField name="KS" fld="21" subtotal="max" baseField="2" baseItem="0" numFmtId="178"/>
   </dataFields>
   <formats count="21">
-    <format dxfId="258">
+    <format dxfId="69">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="257">
+    <format dxfId="68">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="256">
+    <format dxfId="67">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="255">
+    <format dxfId="66">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="254">
+    <format dxfId="65">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="253">
+    <format dxfId="64">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="252">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="251">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="250">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="249">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="248">
+    <format dxfId="59">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="247">
+    <format dxfId="58">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="246">
+    <format dxfId="57">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="245">
+    <format dxfId="56">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="244">
+    <format dxfId="55">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="243">
+    <format dxfId="54">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="242">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="241">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="240">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="239">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="238">
+    <format dxfId="49">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -4889,7 +3774,7 @@
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E1C2EDF3-DA9D-4B5F-A88A-9AED0257874E}" name="数据透视表3" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Feature" colHeaderCaption="Group">
   <location ref="A4:B6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="21">
+  <pivotFields count="22">
     <pivotField axis="axisPage" showAll="0">
       <items count="4">
         <item m="1" x="2"/>
@@ -5070,6 +3955,7 @@
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField numFmtId="177" showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -5095,83 +3981,83 @@
     <dataField name="AUC" fld="17" subtotal="max" baseField="1" baseItem="21" numFmtId="178"/>
   </dataFields>
   <formats count="21">
-    <format dxfId="237">
+    <format dxfId="48">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="236">
+    <format dxfId="47">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="235">
+    <format dxfId="46">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="234">
+    <format dxfId="45">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="233">
+    <format dxfId="44">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="232">
+    <format dxfId="43">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="231">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="230">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="229">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="228">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="227">
+    <format dxfId="38">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="226">
+    <format dxfId="37">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="225">
+    <format dxfId="36">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="224">
+    <format dxfId="35">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="223">
+    <format dxfId="34">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="222">
+    <format dxfId="33">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="221">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="220">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="219">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="218">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="217">
+    <format dxfId="28">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -5188,30 +4074,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73489535-5F3C-4236-A955-4E0C5ACDF166}" name="detail" displayName="detail" ref="A1:U3" totalsRowShown="0" headerRowDxfId="375" dataDxfId="374">
-  <autoFilter ref="A1:U3" xr:uid="{73489535-5F3C-4236-A955-4E0C5ACDF166}"/>
-  <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{847E9846-5D09-4B22-96D7-00A15E265DF1}" name="y" dataDxfId="373"/>
-    <tableColumn id="2" xr3:uid="{A302BC46-C3F8-480A-BCEE-CC2B73F6B6AD}" name="feature" dataDxfId="372"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73489535-5F3C-4236-A955-4E0C5ACDF166}" name="detail" displayName="detail" ref="A1:V3" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+  <autoFilter ref="A1:V3" xr:uid="{73489535-5F3C-4236-A955-4E0C5ACDF166}"/>
+  <tableColumns count="22">
+    <tableColumn id="1" xr3:uid="{847E9846-5D09-4B22-96D7-00A15E265DF1}" name="y" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{A302BC46-C3F8-480A-BCEE-CC2B73F6B6AD}" name="feature" dataDxfId="24"/>
     <tableColumn id="20" xr3:uid="{C31E309C-2FD8-4148-B022-9A791C9E581F}" name="trend"/>
-    <tableColumn id="3" xr3:uid="{15F7C32B-EFFD-41FD-9B31-0FD89CCE1558}" name="mars_group" dataDxfId="371"/>
-    <tableColumn id="4" xr3:uid="{E0412AC0-75F8-47FC-9AFE-DCC4E408E83E}" name="bin_index" dataDxfId="370"/>
-    <tableColumn id="5" xr3:uid="{441B9B96-D32B-4467-BF91-7B8716B0EE73}" name="bin_label" dataDxfId="369"/>
-    <tableColumn id="6" xr3:uid="{7727AFD4-5E39-4798-91A2-841BCB625955}" name="count" dataDxfId="368"/>
-    <tableColumn id="7" xr3:uid="{6904BB63-FC08-4541-9B35-574D79859015}" name="bad" dataDxfId="367"/>
-    <tableColumn id="8" xr3:uid="{A2225E50-387E-446F-9407-B02F0A068262}" name="good" dataDxfId="366"/>
-    <tableColumn id="9" xr3:uid="{350FB9ED-586A-45CB-B3FA-3EECA4545E6F}" name="pct" dataDxfId="365"/>
-    <tableColumn id="10" xr3:uid="{92B3D771-6574-4A45-94E0-F3C28B2BB623}" name="bad_rate" dataDxfId="364"/>
-    <tableColumn id="11" xr3:uid="{0C7A8AE2-4171-40BA-96E5-E18FDDF74290}" name="lift" dataDxfId="363"/>
-    <tableColumn id="12" xr3:uid="{1DB142B5-C1ED-4CEA-BB78-DE1102B6241D}" name="cum_count" dataDxfId="362"/>
-    <tableColumn id="13" xr3:uid="{B7DCD3B6-CA70-4792-909A-DE823943AC34}" name="cum_bad" dataDxfId="361"/>
-    <tableColumn id="14" xr3:uid="{40C7C533-5EAC-4962-87CA-7658DA8C70CB}" name="cum_bad_rate" dataDxfId="360"/>
-    <tableColumn id="15" xr3:uid="{503E378E-7A3D-49D1-A134-2AB9BD4CABEC}" name="psi_bin" dataDxfId="359"/>
-    <tableColumn id="16" xr3:uid="{C6917BCE-A605-4BC0-8F8E-7C3EF22C93C7}" name="ks_bin" dataDxfId="358"/>
-    <tableColumn id="17" xr3:uid="{C37BE33F-0EDB-4EF8-92F6-B944648DE9A6}" name="auc_bin" dataDxfId="357"/>
-    <tableColumn id="18" xr3:uid="{68101AA9-F736-4824-80B4-F4EDB79EA91D}" name="iv_bin" dataDxfId="356"/>
-    <tableColumn id="19" xr3:uid="{0C9E5D86-5C90-4CCE-8D7B-58AB94F13C86}" name="total_count" dataDxfId="355"/>
-    <tableColumn id="21" xr3:uid="{45ABDF0B-7ED1-47FC-8BED-16F072F6736F}" name="bin_type" dataDxfId="354"/>
+    <tableColumn id="3" xr3:uid="{15F7C32B-EFFD-41FD-9B31-0FD89CCE1558}" name="mars_group" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{E0412AC0-75F8-47FC-9AFE-DCC4E408E83E}" name="bin_index" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{441B9B96-D32B-4467-BF91-7B8716B0EE73}" name="bin_label" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{7727AFD4-5E39-4798-91A2-841BCB625955}" name="count" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{6904BB63-FC08-4541-9B35-574D79859015}" name="bad" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{A2225E50-387E-446F-9407-B02F0A068262}" name="good" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{350FB9ED-586A-45CB-B3FA-3EECA4545E6F}" name="pct" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{92B3D771-6574-4A45-94E0-F3C28B2BB623}" name="bad_rate" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{0C7A8AE2-4171-40BA-96E5-E18FDDF74290}" name="lift" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{1DB142B5-C1ED-4CEA-BB78-DE1102B6241D}" name="cum_count" dataDxfId="14"/>
+    <tableColumn id="13" xr3:uid="{B7DCD3B6-CA70-4792-909A-DE823943AC34}" name="cum_bad" dataDxfId="13"/>
+    <tableColumn id="14" xr3:uid="{40C7C533-5EAC-4962-87CA-7658DA8C70CB}" name="cum_bad_rate" dataDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{503E378E-7A3D-49D1-A134-2AB9BD4CABEC}" name="psi_bin" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{C6917BCE-A605-4BC0-8F8E-7C3EF22C93C7}" name="ks_bin" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{C37BE33F-0EDB-4EF8-92F6-B944648DE9A6}" name="auc_bin" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{68101AA9-F736-4824-80B4-F4EDB79EA91D}" name="iv_bin" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{0C9E5D86-5C90-4CCE-8D7B-58AB94F13C86}" name="total_count" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{45ABDF0B-7ED1-47FC-8BED-16F072F6736F}" name="bin_type" dataDxfId="6"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="ks"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5917,9 +4804,7 @@
       <c r="C6" s="28">
         <v>0</v>
       </c>
-      <c r="D6" s="28">
-        <v>0</v>
-      </c>
+      <c r="D6" s="28"/>
       <c r="E6" s="28">
         <v>0</v>
       </c>
@@ -5942,7 +4827,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2">
-    <cfRule type="cellIs" dxfId="216" priority="22" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="22" operator="greaterThan">
       <formula>0.2</formula>
     </cfRule>
     <cfRule type="colorScale" priority="23">
@@ -5957,7 +4842,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" dxfId="215" priority="20" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="20" operator="greaterThan">
       <formula>20</formula>
     </cfRule>
     <cfRule type="colorScale" priority="21">
@@ -5984,7 +4869,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2">
-    <cfRule type="cellIs" dxfId="214" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="18" operator="greaterThan">
       <formula>0.625</formula>
     </cfRule>
     <cfRule type="colorScale" priority="19">
@@ -6358,7 +5243,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C2">
-    <cfRule type="cellIs" dxfId="213" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="greaterThan">
       <formula>0.2</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6429,9 +5314,7 @@
       <c r="A6" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="28">
-        <v>0</v>
-      </c>
+      <c r="B6" s="28"/>
       <c r="C6"/>
     </row>
     <row r="7" spans="1:3" ht="14.25">
@@ -6442,7 +5325,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C2">
-    <cfRule type="cellIs" dxfId="212" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="greaterThan">
       <formula>20</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6525,7 +5408,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C2">
-    <cfRule type="cellIs" dxfId="211" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="greaterThan">
       <formula>0.625</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6545,7 +5428,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr defaultRowHeight="11.25"/>
   <cols>
     <col min="1" max="1" width="4.06640625" style="1" bestFit="1" customWidth="1"/>
@@ -6572,7 +5455,7 @@
     <col min="22" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:22" ht="14.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -6636,8 +5519,11 @@
       <c r="U1" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:21">
+      <c r="V1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6696,7 +5582,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:22">
       <c r="D3" s="3" t="s">
         <v>18</v>
       </c>

</xml_diff>